<commit_message>
Saving rules for Universal OR strategy
</commit_message>
<xml_diff>
--- a/Order_Management.xlsx
+++ b/Order_Management.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohammed Khalid\OneDrive\Desktop\WSGTA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohammed Khalid\OneDrive\Desktop\WSGTA\Github\universal-or-strategy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270091C7-9991-4D4C-A656-6AE5293B3615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D6F581-4B4D-4652-8F4F-95ED29C64246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{443257C1-151D-4D5B-B416-D4B7290BC384}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="128">
   <si>
     <t>Trade</t>
   </si>
@@ -404,13 +404,28 @@
   </si>
   <si>
     <t xml:space="preserve">Add fibs </t>
+  </si>
+  <si>
+    <t>ORB numbers on chart</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>Click</t>
+  </si>
+  <si>
+    <t>when it goes against auto auto break even</t>
+  </si>
+  <si>
+    <t>Apex Compliance:** Strictly enforce rate limiting (max 1 order modification per second) and risk management rules. Is this in the code now rate limiting?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -471,6 +486,27 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -640,7 +676,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -656,17 +692,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -677,9 +707,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -693,10 +720,36 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -706,39 +759,38 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="25">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -965,6 +1017,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1173,20 +1228,20 @@
     <tableColumn id="36" xr3:uid="{2F723897-3760-4B19-AD3B-BCFBA1F3046B}" name="Target 2 " dataDxfId="16"/>
     <tableColumn id="37" xr3:uid="{B0228055-B9F0-4376-9F4B-E5C7ECEC374E}" name="Target 3" dataDxfId="15"/>
     <tableColumn id="17" xr3:uid="{7CC3D155-497E-446B-A522-0C4A9AE7DA8D}" name="BE Trigger" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{5A6E6A7C-0D76-470A-81B6-DC838B39B5C4}" name="BE Offset (t)" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{6FC4F2C6-D6C6-47D3-8D38-72AB148DAFEF}" name="trail1 Trigger (pts)" dataDxfId="13"/>
-    <tableColumn id="16" xr3:uid="{8AA31D74-6B23-44D9-9308-370238BD8AF2}" name="Trail1 Distance (pts)" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{803838AC-CC2F-4B13-BA83-8B235A2B7979}" name="Frequency" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{C8E30A81-9A2B-4FB6-B8DF-121E9D1D8311}" name="Trail2 Trigger (pts)" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{A0CCBB03-A13C-4BC3-9F5E-4DA389FEE99B}" name="Trail2 Distance (pts)" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{005D4A69-D483-4A76-AE2E-EA4663A26F7F}" name="Step 2 Frequency" dataDxfId="8"/>
-    <tableColumn id="14" xr3:uid="{54D8ADB7-AC18-47AE-9CC3-0EB9A0711574}" name="trail3 Trigger (pts)" dataDxfId="7"/>
-    <tableColumn id="19" xr3:uid="{00B2CDE8-9EAA-4C1B-985D-A54CA250F42C}" name="Trail3 Distance (pts)" dataDxfId="6"/>
-    <tableColumn id="20" xr3:uid="{549EE94F-A456-41A9-BD1E-91EF731DFD75}" name="Step 3 Frequency" dataDxfId="5"/>
-    <tableColumn id="35" xr3:uid="{3CC47613-3113-48A8-947D-6BFD5041B252}" name="Direction" dataDxfId="4"/>
-    <tableColumn id="21" xr3:uid="{A81BB64B-3F9E-46D1-8DC6-E7152EFC37AB}" name="Entry Criteria" dataDxfId="3"/>
-    <tableColumn id="22" xr3:uid="{BF3BF641-5A58-4CC8-99E6-52116BA6F0C1}" name="Execution Criteria" dataDxfId="2"/>
-    <tableColumn id="23" xr3:uid="{EDCDBC5F-1F59-4512-81F4-43551DDE86E7}" name="Column1" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{5A6E6A7C-0D76-470A-81B6-DC838B39B5C4}" name="BE Offset (t)" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{6FC4F2C6-D6C6-47D3-8D38-72AB148DAFEF}" name="trail1 Trigger (pts)" dataDxfId="12"/>
+    <tableColumn id="16" xr3:uid="{8AA31D74-6B23-44D9-9308-370238BD8AF2}" name="Trail1 Distance (pts)" dataDxfId="11"/>
+    <tableColumn id="18" xr3:uid="{803838AC-CC2F-4B13-BA83-8B235A2B7979}" name="Frequency" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{C8E30A81-9A2B-4FB6-B8DF-121E9D1D8311}" name="Trail2 Trigger (pts)" dataDxfId="9"/>
+    <tableColumn id="15" xr3:uid="{A0CCBB03-A13C-4BC3-9F5E-4DA389FEE99B}" name="Trail2 Distance (pts)" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{005D4A69-D483-4A76-AE2E-EA4663A26F7F}" name="Step 2 Frequency" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{54D8ADB7-AC18-47AE-9CC3-0EB9A0711574}" name="trail3 Trigger (pts)" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{00B2CDE8-9EAA-4C1B-985D-A54CA250F42C}" name="Trail3 Distance (pts)" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{549EE94F-A456-41A9-BD1E-91EF731DFD75}" name="Step 3 Frequency" dataDxfId="4"/>
+    <tableColumn id="35" xr3:uid="{3CC47613-3113-48A8-947D-6BFD5041B252}" name="Direction" dataDxfId="3"/>
+    <tableColumn id="21" xr3:uid="{A81BB64B-3F9E-46D1-8DC6-E7152EFC37AB}" name="Entry Criteria" dataDxfId="2"/>
+    <tableColumn id="22" xr3:uid="{BF3BF641-5A58-4CC8-99E6-52116BA6F0C1}" name="Execution Criteria" dataDxfId="1"/>
+    <tableColumn id="23" xr3:uid="{EDCDBC5F-1F59-4512-81F4-43551DDE86E7}" name="Column1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1599,595 +1654,567 @@
       <c r="AK1"/>
       <c r="AL1"/>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2" spans="1:38" s="39" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="40">
         <v>0</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="40">
         <v>1</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="40">
         <v>3</v>
       </c>
-      <c r="M2" s="1">
+      <c r="M2" s="40">
         <v>2</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="40">
         <v>2</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="40">
         <v>4</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="40">
         <v>1.5</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="40">
         <v>2</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="40">
         <v>5</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="40">
         <v>1</v>
       </c>
-      <c r="T2" s="1">
+      <c r="T2" s="40">
         <v>1</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="U2" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="7" t="s">
+      <c r="V2" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="W2" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="X2" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="AI2"/>
-      <c r="AJ2"/>
-      <c r="AK2"/>
-      <c r="AL2"/>
-    </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    </row>
+    <row r="3" spans="1:38" s="37" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>0</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>1</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L3" s="2">
         <v>3</v>
       </c>
-      <c r="M3" s="1">
+      <c r="M3" s="2">
         <v>2</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>2</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>4</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>1.5</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>2</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <v>5</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <v>1</v>
       </c>
-      <c r="T3" s="1">
+      <c r="T3" s="2">
         <v>1</v>
       </c>
-      <c r="U3" s="1" t="s">
+      <c r="U3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="V3" s="7" t="s">
+      <c r="V3" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="W3" s="1" t="s">
+      <c r="W3" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="X3" s="1" t="s">
+      <c r="X3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="AI3"/>
-      <c r="AJ3"/>
-      <c r="AK3"/>
-      <c r="AL3"/>
-    </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    </row>
+    <row r="4" spans="1:38" s="42" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="43">
         <v>0</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="43">
         <v>1</v>
       </c>
-      <c r="L4" s="1">
+      <c r="L4" s="43">
         <v>3</v>
       </c>
-      <c r="M4" s="1">
+      <c r="M4" s="43">
         <v>2</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="43">
         <v>2</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="43">
         <v>4</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="43">
         <v>1.5</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="43">
         <v>2</v>
       </c>
-      <c r="R4" s="1">
+      <c r="R4" s="43">
         <v>5</v>
       </c>
-      <c r="S4" s="1">
+      <c r="S4" s="43">
         <v>1</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="43">
         <v>1</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="U4" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="V4" s="7" t="s">
+      <c r="V4" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="W4" s="1" t="s">
+      <c r="W4" s="43" t="s">
         <v>91</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="X4" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="AI4"/>
-      <c r="AJ4"/>
-      <c r="AK4"/>
-      <c r="AL4"/>
-    </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    </row>
+    <row r="5" spans="1:38" s="34" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="35">
         <v>2</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="35">
         <v>1</v>
       </c>
-      <c r="L5" s="1">
+      <c r="L5" s="35">
         <v>3</v>
       </c>
-      <c r="M5" s="1">
+      <c r="M5" s="35">
         <v>2</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="35">
         <v>2</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="35">
         <v>4</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="35">
         <v>1.5</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="35">
         <v>2</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="35">
         <v>5</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="35">
         <v>1</v>
       </c>
-      <c r="T5" s="1">
+      <c r="T5" s="35">
         <v>1</v>
       </c>
-      <c r="U5" s="1" t="s">
+      <c r="U5" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="V5" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="W5" s="1" t="s">
+      <c r="W5" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="X5" s="1" t="s">
+      <c r="X5" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="AI5"/>
-      <c r="AJ5"/>
-      <c r="AK5"/>
-      <c r="AL5"/>
-    </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+    </row>
+    <row r="6" spans="1:38" s="37" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="2">
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>1</v>
       </c>
-      <c r="L6" s="1">
+      <c r="L6" s="2">
         <v>3</v>
       </c>
-      <c r="M6" s="1">
+      <c r="M6" s="2">
         <v>2</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>2</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>4</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>1.5</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>2</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <v>5</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <v>1</v>
       </c>
-      <c r="T6" s="1">
+      <c r="T6" s="2">
         <v>1</v>
       </c>
-      <c r="U6" s="1" t="s">
+      <c r="U6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="V6" s="7" t="s">
+      <c r="V6" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="W6" s="1" t="s">
+      <c r="W6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="X6" s="1" t="s">
+      <c r="X6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="AI6"/>
-      <c r="AJ6"/>
-      <c r="AK6"/>
-      <c r="AL6"/>
-    </row>
-    <row r="7" spans="1:38" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+    </row>
+    <row r="7" spans="1:38" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="8">
         <v>3</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="J7" s="8" t="s">
         <v>52</v>
       </c>
       <c r="K7" s="1">
         <v>1</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="8">
         <v>3</v>
       </c>
-      <c r="M7" s="9">
+      <c r="M7" s="8">
         <v>2</v>
       </c>
-      <c r="N7" s="9">
+      <c r="N7" s="8">
         <v>2</v>
       </c>
-      <c r="O7" s="9">
+      <c r="O7" s="8">
         <v>4</v>
       </c>
-      <c r="P7" s="9">
+      <c r="P7" s="8">
         <v>1.5</v>
       </c>
-      <c r="Q7" s="9">
+      <c r="Q7" s="8">
         <v>2</v>
       </c>
-      <c r="R7" s="9">
+      <c r="R7" s="8">
         <v>5</v>
       </c>
-      <c r="S7" s="9">
+      <c r="S7" s="8">
         <v>1</v>
       </c>
-      <c r="T7" s="9">
+      <c r="T7" s="8">
         <v>1</v>
       </c>
-      <c r="U7" s="9" t="s">
+      <c r="U7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="V7" s="10" t="s">
+      <c r="V7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="W7" s="9" t="s">
+      <c r="W7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="X7" s="9" t="s">
+      <c r="X7" s="8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+    <row r="8" spans="1:38" s="39" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="40">
         <v>0</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="40">
         <v>1</v>
       </c>
-      <c r="L8" s="1">
+      <c r="L8" s="40">
         <v>3</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="40">
         <v>2</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="40">
         <v>2</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="40">
         <v>4</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="40">
         <v>1.5</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="40">
         <v>2</v>
       </c>
-      <c r="R8" s="1">
+      <c r="R8" s="40">
         <v>5</v>
       </c>
-      <c r="S8" s="1">
+      <c r="S8" s="40">
         <v>1</v>
       </c>
-      <c r="T8" s="1">
+      <c r="T8" s="40">
         <v>1</v>
       </c>
-      <c r="U8" s="1" t="s">
+      <c r="U8" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="V8" s="7" t="s">
+      <c r="V8" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="W8" s="1" t="s">
+      <c r="W8" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="X8" s="1" t="s">
+      <c r="X8" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="AI8"/>
-      <c r="AJ8"/>
-      <c r="AK8"/>
-      <c r="AL8"/>
-    </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+    </row>
+    <row r="9" spans="1:38" s="37" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="2">
         <v>0</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>1</v>
       </c>
-      <c r="L9" s="1">
+      <c r="L9" s="2">
         <v>3</v>
       </c>
-      <c r="M9" s="1">
+      <c r="M9" s="2">
         <v>2</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>2</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>4</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>1.5</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>2</v>
       </c>
-      <c r="R9" s="1">
+      <c r="R9" s="2">
         <v>5</v>
       </c>
-      <c r="S9" s="1">
+      <c r="S9" s="2">
         <v>1</v>
       </c>
-      <c r="T9" s="1">
+      <c r="T9" s="2">
         <v>1</v>
       </c>
-      <c r="U9" s="1" t="s">
+      <c r="U9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="V9" s="7" t="s">
+      <c r="V9" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="W9" s="1" t="s">
+      <c r="W9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="X9" s="1" t="s">
+      <c r="X9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="AI9"/>
-      <c r="AJ9"/>
-      <c r="AK9"/>
-      <c r="AL9"/>
     </row>
     <row r="13" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -2253,13 +2280,24 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>123</v>
+      </c>
       <c r="C26" t="s">
         <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C27" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
         <v>69</v>
+      </c>
+      <c r="C28" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -2344,226 +2382,215 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A37874B-405E-42F6-A097-C7A8365BB04E}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="49.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" style="17" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" style="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.36328125" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="15" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="20" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:5" ht="20" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="25"/>
-    </row>
-    <row r="2" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="13" t="s">
+      <c r="C1" s="28"/>
+      <c r="D1" s="21" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-    </row>
-    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="13" t="s">
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+    </row>
+    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="32"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="13"/>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-    </row>
-    <row r="7" spans="1:6" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="13"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
+      <c r="C5" s="30"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="11"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+    </row>
+    <row r="7" spans="1:5" s="10" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="11"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="13" t="s">
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-    </row>
-    <row r="10" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="13" t="s">
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+    </row>
+    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="14"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="14"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="13" t="s">
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="12"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="12"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="15" t="s">
+      <c r="C13" s="32"/>
+      <c r="D13" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="E13" s="14"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="C14" s="32"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="17">
         <v>9</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="17">
         <v>15</v>
       </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="13" t="s">
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="15" t="s">
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="13"/>
-      <c r="B18" s="26" t="s">
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="11"/>
+      <c r="B18" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="26"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C18" s="31"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>36</v>
       </c>

</xml_diff>